<commit_message>
Słup w zakresie stacji nie jest łączony ze słupem z zakresu innej stacji
</commit_message>
<xml_diff>
--- a/zestawienie pw.xlsx
+++ b/zestawienie pw.xlsx
@@ -245,11 +245,11 @@
       </c>
       <c r="B12">
         <f>COUNTA('05-0918'!A:A)-1</f>
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C12">
         <f>SUM('05-0918'!D:D)</f>
-        <v>1778</v>
+        <v>1815</v>
       </c>
     </row>
     <row r="13">
@@ -260,11 +260,11 @@
       </c>
       <c r="B13">
         <f>COUNTA('05-1067'!A:A)-1</f>
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C13">
         <f>SUM('05-1067'!D:D)</f>
-        <v>796</v>
+        <v>769</v>
       </c>
     </row>
     <row r="14">
@@ -294,7 +294,7 @@
       </c>
       <c r="C15">
         <f>SUM(C2:C14)</f>
-        <v>12585</v>
+        <v>12595</v>
       </c>
     </row>
   </sheetData>
@@ -2543,6 +2543,29 @@
         <v>3</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kr</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-10/ZN</t>
+        </is>
+      </c>
+      <c r="D51">
+        <v>37</v>
+      </c>
+      <c r="F51">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -2835,12 +2858,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">12</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kr</t>
+          <t xml:space="preserve">Or</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2852,18 +2875,18 @@
         <v>27</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Or</t>
+          <t xml:space="preserve">RPKr</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2872,7 +2895,7 @@
         </is>
       </c>
       <c r="D13">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="F13">
         <v>2</v>
@@ -2881,7 +2904,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2895,7 +2918,10 @@
         </is>
       </c>
       <c r="D14">
-        <v>41</v>
+        <v>37</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
       </c>
       <c r="F14">
         <v>2</v>
@@ -2904,12 +2930,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">3.1</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">RPKr</t>
+          <t xml:space="preserve">P</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2918,10 +2944,7 @@
         </is>
       </c>
       <c r="D15">
-        <v>37</v>
-      </c>
-      <c r="E15">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="F15">
         <v>2</v>
@@ -2930,7 +2953,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.1</t>
+          <t xml:space="preserve">3.2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2944,7 +2967,7 @@
         </is>
       </c>
       <c r="D16">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="F16">
         <v>2</v>
@@ -2953,12 +2976,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.2</t>
+          <t xml:space="preserve">3.3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">P</t>
+          <t xml:space="preserve">Kr</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2967,7 +2990,10 @@
         </is>
       </c>
       <c r="D17">
-        <v>49</v>
+        <v>46</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
       </c>
       <c r="F17">
         <v>2</v>
@@ -2976,12 +3002,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.3</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kr</t>
+          <t xml:space="preserve">P</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2990,10 +3016,7 @@
         </is>
       </c>
       <c r="D18">
-        <v>46</v>
-      </c>
-      <c r="E18">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="F18">
         <v>2</v>
@@ -3002,12 +3025,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">P</t>
+          <t xml:space="preserve">Nr</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3016,7 +3039,7 @@
         </is>
       </c>
       <c r="D19">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="F19">
         <v>2</v>
@@ -3025,12 +3048,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nr</t>
+          <t xml:space="preserve">Kr</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3039,32 +3062,9 @@
         </is>
       </c>
       <c r="D20">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="F20">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kr</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-10/ZN</t>
-        </is>
-      </c>
-      <c r="D21">
-        <v>40</v>
-      </c>
-      <c r="F21">
         <v>2</v>
       </c>
     </row>
@@ -4050,7 +4050,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stacja 05-1067, obwód 1: jest słup nr 12, a brak słupa nr 11 (luka w numeracji?).</t>
+          <t xml:space="preserve">Słup nr 12 (7549433.68, 5784553.36): brak wymiaru - odległość zmierzona geometrycznie (37 m).</t>
         </is>
       </c>
     </row>

</xml_diff>